<commit_message>
Add Summary sheet: 27 unique compounds vs 64 memberships listed
New first sheet states the unique-compound count, total compound-pathway
memberships (with repeats), and lists each unique compound with how many
pathways it spans + duplicate-molecule notes. Clarifies why the per-pathway
view shows ~64 cells while there are 27 distinct compounds.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pathway-mapping/pathway-membership.xlsx
+++ b/pathway-mapping/pathway-membership.xlsx
@@ -4,17 +4,345 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Pathways → Compounds" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Compound detail" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Coverage gaps" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Methods &amp; changelog" state="visible" r:id="rId7"/>
+    <sheet sheetId="1" name="Summary" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Pathways → Compounds" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Compound detail" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Coverage gaps" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Methods &amp; changelog" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="218">
+  <si>
+    <t>Elderberry compounds mapped to the 13 enriched SMPDB pathways</t>
+  </si>
+  <si>
+    <t>Unique compounds:</t>
+  </si>
+  <si>
+    <t>Memberships listed across the 13 pathways:</t>
+  </si>
+  <si>
+    <t>(each compound is listed once per pathway it belongs to — hub metabolites like glutamate &amp; alpha-ketoglutarate span many, so memberships &gt; unique)</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Unique compound</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>PubChem CID</t>
+  </si>
+  <si>
+    <t># pathways</t>
+  </si>
+  <si>
+    <t>Pathways it appears in</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>DL-Glutamic acid</t>
+  </si>
+  <si>
+    <t>C5H9NO4</t>
+  </si>
+  <si>
+    <t>611</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Beta-Alanine Metabolism; Aspartate Metabolism; Valine, Leucine and Isoleucine Degradation; Phenylalanine and Tyrosine Metabolism; Malate-Aspartate Shuttle; Arginine and Proline Metabolism; Amino Sugar Metabolism; Glycine and Serine Metabolism</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>L-Glutamate</t>
+  </si>
+  <si>
+    <t>33032</t>
+  </si>
+  <si>
+    <t>same molecule as: L-Glutamic acid</t>
+  </si>
+  <si>
+    <t>L-Glutamic acid</t>
+  </si>
+  <si>
+    <t>same molecule as: L-Glutamate</t>
+  </si>
+  <si>
+    <t>alpha-Ketoglutaric acid</t>
+  </si>
+  <si>
+    <t>C5H6O5</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Beta-Alanine Metabolism; Aspartate Metabolism; Valine, Leucine and Isoleucine Degradation; Phenylalanine and Tyrosine Metabolism; Malate-Aspartate Shuttle; Arginine and Proline Metabolism; Glycine and Serine Metabolism</t>
+  </si>
+  <si>
+    <t>Serine</t>
+  </si>
+  <si>
+    <t>C3H7NO3</t>
+  </si>
+  <si>
+    <t>5951</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Methionine Metabolism; Phosphatidylethanolamine Biosynthesis; Glycine and Serine Metabolism; Homocysteine Degradation</t>
+  </si>
+  <si>
+    <t>Arginine</t>
+  </si>
+  <si>
+    <t>C6H14N4O2</t>
+  </si>
+  <si>
+    <t>6322</t>
+  </si>
+  <si>
+    <t>Aspartate Metabolism; Arginine and Proline Metabolism; Glycine and Serine Metabolism</t>
+  </si>
+  <si>
+    <t>Choline</t>
+  </si>
+  <si>
+    <t>C5H13NO</t>
+  </si>
+  <si>
+    <t>305</t>
+  </si>
+  <si>
+    <t>Methionine Metabolism; Phosphatidylethanolamine Biosynthesis; Betaine Metabolism</t>
+  </si>
+  <si>
+    <t>Glutamine</t>
+  </si>
+  <si>
+    <t>C5H10N2O3</t>
+  </si>
+  <si>
+    <t>5961</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Aspartate Metabolism; Amino Sugar Metabolism</t>
+  </si>
+  <si>
+    <t>Methionine</t>
+  </si>
+  <si>
+    <t>C5H11NO2S</t>
+  </si>
+  <si>
+    <t>6137</t>
+  </si>
+  <si>
+    <t>Methionine Metabolism; Glycine and Serine Metabolism; Betaine Metabolism</t>
+  </si>
+  <si>
+    <t>Asparagine</t>
+  </si>
+  <si>
+    <t>C4H8N2O3</t>
+  </si>
+  <si>
+    <t>6267</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Aspartate Metabolism</t>
+  </si>
+  <si>
+    <t>Histidine</t>
+  </si>
+  <si>
+    <t>C6H9N3O2</t>
+  </si>
+  <si>
+    <t>6274</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Beta-Alanine Metabolism</t>
+  </si>
+  <si>
+    <t>L-Pyroglutamic acid/5-Oxo-proline</t>
+  </si>
+  <si>
+    <t>C5H7NO3</t>
+  </si>
+  <si>
+    <t>7405</t>
+  </si>
+  <si>
+    <t>Ammonia Recycling; Arginine and Proline Metabolism</t>
+  </si>
+  <si>
+    <t>5-Aminolevulinic acid</t>
+  </si>
+  <si>
+    <t>C5H9NO3</t>
+  </si>
+  <si>
+    <t>137</t>
+  </si>
+  <si>
+    <t>Glycine and Serine Metabolism</t>
+  </si>
+  <si>
+    <t>Adenosine</t>
+  </si>
+  <si>
+    <t>C10H13N5O4</t>
+  </si>
+  <si>
+    <t>60961</t>
+  </si>
+  <si>
+    <t>Betaine Metabolism</t>
+  </si>
+  <si>
+    <t>cis-4-Hydroxy-D-proline</t>
+  </si>
+  <si>
+    <t>440014</t>
+  </si>
+  <si>
+    <t>Arginine and Proline Metabolism</t>
+  </si>
+  <si>
+    <t>Cytidine</t>
+  </si>
+  <si>
+    <t>C9H13N3O5</t>
+  </si>
+  <si>
+    <t>6175</t>
+  </si>
+  <si>
+    <t>Phosphatidylethanolamine Biosynthesis</t>
+  </si>
+  <si>
+    <t>D-Pantothenic acid</t>
+  </si>
+  <si>
+    <t>C9H17NO5</t>
+  </si>
+  <si>
+    <t>6613</t>
+  </si>
+  <si>
+    <t>Beta-Alanine Metabolism</t>
+  </si>
+  <si>
+    <t>H-Met(O)-OH</t>
+  </si>
+  <si>
+    <t>C5H11NO3S</t>
+  </si>
+  <si>
+    <t>158980</t>
+  </si>
+  <si>
+    <t>Methionine Metabolism</t>
+  </si>
+  <si>
+    <t>Isoleucine</t>
+  </si>
+  <si>
+    <t>C6H13NO2</t>
+  </si>
+  <si>
+    <t>6306</t>
+  </si>
+  <si>
+    <t>Valine, Leucine and Isoleucine Degradation</t>
+  </si>
+  <si>
+    <t>Leucine</t>
+  </si>
+  <si>
+    <t>6106</t>
+  </si>
+  <si>
+    <t>N-Acetylglucosaminitol</t>
+  </si>
+  <si>
+    <t>C8H17NO6</t>
+  </si>
+  <si>
+    <t>165206</t>
+  </si>
+  <si>
+    <t>Amino Sugar Metabolism</t>
+  </si>
+  <si>
+    <t>Phenylalanine</t>
+  </si>
+  <si>
+    <t>C9H11NO2</t>
+  </si>
+  <si>
+    <t>6140</t>
+  </si>
+  <si>
+    <t>Phenylalanine and Tyrosine Metabolism</t>
+  </si>
+  <si>
+    <t>phosphoethanolamine</t>
+  </si>
+  <si>
+    <t>C2H8NO4P</t>
+  </si>
+  <si>
+    <t>1015</t>
+  </si>
+  <si>
+    <t>Proline</t>
+  </si>
+  <si>
+    <t>C5H9NO2</t>
+  </si>
+  <si>
+    <t>145742</t>
+  </si>
+  <si>
+    <t>Spermidine</t>
+  </si>
+  <si>
+    <t>C7H19N3</t>
+  </si>
+  <si>
+    <t>1102</t>
+  </si>
+  <si>
+    <t>Tyrosine</t>
+  </si>
+  <si>
+    <t>C9H11NO3</t>
+  </si>
+  <si>
+    <t>6057</t>
+  </si>
+  <si>
+    <t>Valine</t>
+  </si>
+  <si>
+    <t>C5H11NO2</t>
+  </si>
+  <si>
+    <t>6287</t>
+  </si>
   <si>
     <t>Pathway</t>
   </si>
@@ -55,141 +383,39 @@
     <t>Both (Conventional + Organic)</t>
   </si>
   <si>
-    <t>alpha-Ketoglutaric acid</t>
-  </si>
-  <si>
-    <t>Asparagine</t>
-  </si>
-  <si>
-    <t>DL-Glutamic acid</t>
-  </si>
-  <si>
-    <t>Glutamine</t>
-  </si>
-  <si>
-    <t>Histidine</t>
-  </si>
-  <si>
     <t>L-Glutamate [+1 dup]</t>
   </si>
   <si>
-    <t>Serine</t>
-  </si>
-  <si>
     <t>L-Pyroglutamic acid/5-Oxo-proline (low·stereo/parent)</t>
   </si>
   <si>
-    <t>Beta-Alanine Metabolism</t>
-  </si>
-  <si>
     <t>GAP Conventional vs No GAP</t>
   </si>
   <si>
-    <t>D-Pantothenic acid</t>
-  </si>
-  <si>
     <t>Aspartate Metabolism</t>
   </si>
   <si>
-    <t>Arginine</t>
-  </si>
-  <si>
-    <t>Valine, Leucine and Isoleucine Degradation</t>
-  </si>
-  <si>
-    <t>Isoleucine</t>
-  </si>
-  <si>
-    <t>Leucine</t>
-  </si>
-  <si>
-    <t>Valine</t>
-  </si>
-  <si>
-    <t>Phenylalanine and Tyrosine Metabolism</t>
-  </si>
-  <si>
-    <t>Phenylalanine</t>
-  </si>
-  <si>
-    <t>Tyrosine</t>
-  </si>
-  <si>
     <t>Malate-Aspartate Shuttle</t>
   </si>
   <si>
-    <t>Arginine and Proline Metabolism</t>
-  </si>
-  <si>
-    <t>cis-4-Hydroxy-D-proline</t>
-  </si>
-  <si>
-    <t>Proline</t>
-  </si>
-  <si>
-    <t>Amino Sugar Metabolism</t>
-  </si>
-  <si>
     <t>N-Acetylglucosaminitol (low·stereo/parent)</t>
   </si>
   <si>
-    <t>Methionine Metabolism</t>
-  </si>
-  <si>
     <t>GAP Organic vs No GAP</t>
   </si>
   <si>
-    <t>Choline</t>
-  </si>
-  <si>
-    <t>H-Met(O)-OH</t>
-  </si>
-  <si>
-    <t>Methionine</t>
-  </si>
-  <si>
-    <t>Spermidine</t>
-  </si>
-  <si>
-    <t>Phosphatidylethanolamine Biosynthesis</t>
-  </si>
-  <si>
-    <t>phosphoethanolamine</t>
-  </si>
-  <si>
     <t>Cytidine (low·stereo/parent)</t>
   </si>
   <si>
-    <t>Glycine and Serine Metabolism</t>
-  </si>
-  <si>
-    <t>5-Aminolevulinic acid</t>
-  </si>
-  <si>
-    <t>Betaine Metabolism</t>
-  </si>
-  <si>
-    <t>Adenosine</t>
-  </si>
-  <si>
     <t>Homocysteine Degradation</t>
   </si>
   <si>
     <t>Name</t>
   </si>
   <si>
-    <t>Formula</t>
-  </si>
-  <si>
-    <t>PubChem CID</t>
-  </si>
-  <si>
     <t>InChIKey</t>
   </si>
   <si>
-    <t># pathways</t>
-  </si>
-  <si>
     <t>Pathways</t>
   </si>
   <si>
@@ -208,12 +434,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>C5H9NO3</t>
-  </si>
-  <si>
-    <t>137</t>
-  </si>
-  <si>
     <t>ZGXJTSGNIOSYLO-UHFFFAOYSA-N</t>
   </si>
   <si>
@@ -223,81 +443,24 @@
     <t>high</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>C10H13N5O4</t>
-  </si>
-  <si>
-    <t>60961</t>
-  </si>
-  <si>
     <t>OIRDTQYFTABQOQ-KQYNXXCUSA-N</t>
   </si>
   <si>
-    <t>C5H6O5</t>
-  </si>
-  <si>
-    <t>51</t>
-  </si>
-  <si>
     <t>KPGXRSRHYNQIFN-UHFFFAOYSA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Beta-Alanine Metabolism; Aspartate Metabolism; Valine, Leucine and Isoleucine Degradation; Phenylalanine and Tyrosine Metabolism; Malate-Aspartate Shuttle; Arginine and Proline Metabolism; Glycine and Serine Metabolism</t>
-  </si>
-  <si>
-    <t>C6H14N4O2</t>
-  </si>
-  <si>
-    <t>6322</t>
-  </si>
-  <si>
     <t>ODKSFYDXXFIFQN-BYPYZUCNSA-N</t>
   </si>
   <si>
-    <t>Aspartate Metabolism; Arginine and Proline Metabolism; Glycine and Serine Metabolism</t>
-  </si>
-  <si>
-    <t>C4H8N2O3</t>
-  </si>
-  <si>
-    <t>6267</t>
-  </si>
-  <si>
     <t>DCXYFEDJOCDNAF-REOHCLBHSA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Aspartate Metabolism</t>
-  </si>
-  <si>
-    <t>C5H13NO</t>
-  </si>
-  <si>
-    <t>305</t>
-  </si>
-  <si>
     <t>OEYIOHPDSNJKLS-UHFFFAOYSA-N</t>
   </si>
   <si>
-    <t>Methionine Metabolism; Phosphatidylethanolamine Biosynthesis; Betaine Metabolism</t>
-  </si>
-  <si>
-    <t>440014</t>
-  </si>
-  <si>
     <t>PMMYEEVYMWASQN-QWWZWVQMSA-N</t>
   </si>
   <si>
-    <t>Cytidine</t>
-  </si>
-  <si>
-    <t>C9H13N3O5</t>
-  </si>
-  <si>
-    <t>6175</t>
-  </si>
-  <si>
     <t>UHDGCWIWMRVCDJ-XVFCMESISA-N</t>
   </si>
   <si>
@@ -307,187 +470,55 @@
     <t>low</t>
   </si>
   <si>
-    <t>C9H17NO5</t>
-  </si>
-  <si>
-    <t>6613</t>
-  </si>
-  <si>
     <t>GHOKWGTUZJEAQD-ZETCQYMHSA-N</t>
   </si>
   <si>
-    <t>C5H9NO4</t>
-  </si>
-  <si>
-    <t>611</t>
-  </si>
-  <si>
     <t>WHUUTDBJXJRKMK-UHFFFAOYSA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Beta-Alanine Metabolism; Aspartate Metabolism; Valine, Leucine and Isoleucine Degradation; Phenylalanine and Tyrosine Metabolism; Malate-Aspartate Shuttle; Arginine and Proline Metabolism; Amino Sugar Metabolism; Glycine and Serine Metabolism</t>
-  </si>
-  <si>
-    <t>C5H10N2O3</t>
-  </si>
-  <si>
-    <t>5961</t>
-  </si>
-  <si>
     <t>ZDXPYRJPNDTMRX-VKHMYHEASA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Aspartate Metabolism; Amino Sugar Metabolism</t>
-  </si>
-  <si>
-    <t>C5H11NO3S</t>
-  </si>
-  <si>
-    <t>158980</t>
-  </si>
-  <si>
     <t>QEFRNWWLZKMPFJ-YGVKFDHGSA-N</t>
   </si>
   <si>
-    <t>C6H9N3O2</t>
-  </si>
-  <si>
-    <t>6274</t>
-  </si>
-  <si>
     <t>HNDVDQJCIGZPNO-YFKPBYRVSA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Beta-Alanine Metabolism</t>
-  </si>
-  <si>
-    <t>C6H13NO2</t>
-  </si>
-  <si>
-    <t>6306</t>
-  </si>
-  <si>
     <t>AGPKZVBTJJNPAG-WHFBIAKZSA-N</t>
   </si>
   <si>
-    <t>L-Glutamate</t>
-  </si>
-  <si>
-    <t>33032</t>
-  </si>
-  <si>
     <t>WHUUTDBJXJRKMK-VKHMYHEASA-N</t>
   </si>
   <si>
-    <t>L-Glutamic acid</t>
-  </si>
-  <si>
-    <t>L-Pyroglutamic acid/5-Oxo-proline</t>
-  </si>
-  <si>
-    <t>C5H7NO3</t>
-  </si>
-  <si>
-    <t>7405</t>
-  </si>
-  <si>
     <t>ODHCTXKNWHHXJC-VKHMYHEASA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Arginine and Proline Metabolism</t>
-  </si>
-  <si>
-    <t>6106</t>
-  </si>
-  <si>
     <t>ROHFNLRQFUQHCH-YFKPBYRVSA-N</t>
   </si>
   <si>
-    <t>C5H11NO2S</t>
-  </si>
-  <si>
-    <t>6137</t>
-  </si>
-  <si>
     <t>FFEARJCKVFRZRR-BYPYZUCNSA-N</t>
   </si>
   <si>
-    <t>Methionine Metabolism; Glycine and Serine Metabolism; Betaine Metabolism</t>
-  </si>
-  <si>
-    <t>N-Acetylglucosaminitol</t>
-  </si>
-  <si>
-    <t>C8H17NO6</t>
-  </si>
-  <si>
-    <t>165206</t>
-  </si>
-  <si>
     <t>DWAICOVNOFPYLS-LXGUWJNJSA-N</t>
   </si>
   <si>
-    <t>C9H11NO2</t>
-  </si>
-  <si>
-    <t>6140</t>
-  </si>
-  <si>
     <t>COLNVLDHVKWLRT-QMMMGPOBSA-N</t>
   </si>
   <si>
-    <t>C2H8NO4P</t>
-  </si>
-  <si>
-    <t>1015</t>
-  </si>
-  <si>
     <t>SUHOOTKUPISOBE-UHFFFAOYSA-N</t>
   </si>
   <si>
-    <t>C5H9NO2</t>
-  </si>
-  <si>
-    <t>145742</t>
-  </si>
-  <si>
     <t>ONIBWKKTOPOVIA-BYPYZUCNSA-N</t>
   </si>
   <si>
-    <t>C3H7NO3</t>
-  </si>
-  <si>
-    <t>5951</t>
-  </si>
-  <si>
     <t>MTCFGRXMJLQNBG-REOHCLBHSA-N</t>
   </si>
   <si>
-    <t>Ammonia Recycling; Methionine Metabolism; Phosphatidylethanolamine Biosynthesis; Glycine and Serine Metabolism; Homocysteine Degradation</t>
-  </si>
-  <si>
-    <t>C7H19N3</t>
-  </si>
-  <si>
-    <t>1102</t>
-  </si>
-  <si>
     <t>ATHGHQPFGPMSJY-UHFFFAOYSA-N</t>
   </si>
   <si>
-    <t>C9H11NO3</t>
-  </si>
-  <si>
-    <t>6057</t>
-  </si>
-  <si>
     <t>OUYCCCASQSFEME-QMMMGPOBSA-N</t>
-  </si>
-  <si>
-    <t>C5H11NO2</t>
-  </si>
-  <si>
-    <t>6287</t>
   </si>
   <si>
     <t>KZSNJWFQEVHDMF-BYPYZUCNSA-N</t>
@@ -659,13 +690,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
     </font>
     <font>
       <b/>
@@ -691,9 +726,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1033,6 +1069,696 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G34"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="60" customWidth="1"/>
+    <col min="7" max="7" width="38" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8">
+        <v>9</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10">
+        <v>9</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+      <c r="F19" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>60</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>67</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>16</v>
+      </c>
+      <c r="B23" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>71</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>75</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25" t="s">
+        <v>79</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>19</v>
+      </c>
+      <c r="B26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>83</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>20</v>
+      </c>
+      <c r="B27" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" t="s">
+        <v>81</v>
+      </c>
+      <c r="D27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>83</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>21</v>
+      </c>
+      <c r="B28" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
+        <v>89</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>22</v>
+      </c>
+      <c r="B29" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" t="s">
+        <v>92</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29" t="s">
+        <v>93</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>23</v>
+      </c>
+      <c r="B30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>24</v>
+      </c>
+      <c r="B31" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31" t="s">
+        <v>67</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>25</v>
+      </c>
+      <c r="B32" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32" t="s">
+        <v>79</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>26</v>
+      </c>
+      <c r="B33" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" t="s">
+        <v>105</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" t="s">
+        <v>93</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>27</v>
+      </c>
+      <c r="B34" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
+        <v>83</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1042,374 +1768,374 @@
     <col min="4" max="11" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="C2">
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="K2" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>124</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>124</v>
       </c>
       <c r="C4">
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="I4" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>124</v>
       </c>
       <c r="C5">
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="I5" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>124</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
-        <v>32</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>126</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>124</v>
       </c>
       <c r="C7">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>124</v>
       </c>
       <c r="C8">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="I8" t="s">
-        <v>36</v>
+        <v>97</v>
       </c>
       <c r="J8" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="C9">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="G9" t="s">
-        <v>38</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="C10">
         <v>5</v>
       </c>
       <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
         <v>41</v>
       </c>
-      <c r="E10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" t="s">
-        <v>43</v>
-      </c>
       <c r="G10" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H10" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="C11">
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>94</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>47</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="C12">
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F12" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" t="s">
+        <v>122</v>
+      </c>
+      <c r="I12" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" t="s">
         <v>25</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I12" t="s">
-        <v>43</v>
-      </c>
-      <c r="J12" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
         <v>41</v>
-      </c>
-      <c r="F13" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1418,7 +2144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1429,984 +2155,984 @@
     <col min="9" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>63</v>
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>139</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J2" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="G3" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H3" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J3" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="E4">
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J4" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K4" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>79</v>
+        <v>144</v>
       </c>
       <c r="E5">
         <v>3</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H5" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J5" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K5" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="E6">
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J6" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K6" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J7" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K7" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
-        <v>90</v>
+        <v>147</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H8" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K8" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>148</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="G9" t="s">
-        <v>95</v>
+        <v>149</v>
       </c>
       <c r="H9" t="s">
-        <v>96</v>
+        <v>150</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K9" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>99</v>
+        <v>151</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="G10" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K10" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>101</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
       <c r="E11">
         <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H11" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K11" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>106</v>
+        <v>153</v>
       </c>
       <c r="E12">
         <v>3</v>
       </c>
       <c r="F12" t="s">
-        <v>107</v>
+        <v>40</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H12" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K12" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>154</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="G13" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I13" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K13" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>112</v>
+        <v>51</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>155</v>
       </c>
       <c r="E14">
         <v>2</v>
       </c>
       <c r="F14" t="s">
-        <v>114</v>
+        <v>52</v>
       </c>
       <c r="G14" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H14" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I14" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J14" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="D15" t="s">
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="E15">
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H15" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I15" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J15" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K15" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>119</v>
+        <v>17</v>
       </c>
       <c r="D16" t="s">
-        <v>120</v>
+        <v>157</v>
       </c>
       <c r="E16">
         <v>9</v>
       </c>
       <c r="F16" t="s">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H16" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I16" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J16" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K16" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>119</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>120</v>
+        <v>157</v>
       </c>
       <c r="E17">
         <v>9</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H17" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I17" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J17" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K17" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>122</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>123</v>
+        <v>54</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>55</v>
       </c>
       <c r="D18" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18" t="s">
-        <v>126</v>
+        <v>56</v>
       </c>
       <c r="G18" t="s">
-        <v>95</v>
+        <v>149</v>
       </c>
       <c r="H18" t="s">
-        <v>96</v>
+        <v>150</v>
       </c>
       <c r="I18" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J18" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K18" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="D19" t="s">
-        <v>128</v>
+        <v>159</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H19" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I19" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J19" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K19" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" t="s">
         <v>43</v>
       </c>
-      <c r="B20" t="s">
-        <v>129</v>
-      </c>
-      <c r="C20" t="s">
-        <v>130</v>
-      </c>
       <c r="D20" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="E20">
         <v>3</v>
       </c>
       <c r="F20" t="s">
-        <v>132</v>
+        <v>44</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H20" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I20" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J20" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K20" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>133</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>134</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
-        <v>135</v>
+        <v>88</v>
       </c>
       <c r="D21" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="G21" t="s">
-        <v>95</v>
+        <v>149</v>
       </c>
       <c r="H21" t="s">
-        <v>96</v>
+        <v>150</v>
       </c>
       <c r="I21" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J21" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K21" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>90</v>
       </c>
       <c r="B22" t="s">
-        <v>137</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>138</v>
+        <v>92</v>
       </c>
       <c r="D22" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="G22" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H22" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I22" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J22" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K22" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>94</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>95</v>
       </c>
       <c r="C23" t="s">
-        <v>141</v>
+        <v>96</v>
       </c>
       <c r="D23" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="G23" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H23" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I23" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J23" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K23" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>97</v>
       </c>
       <c r="B24" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
       <c r="C24" t="s">
-        <v>144</v>
+        <v>99</v>
       </c>
       <c r="D24" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="G24" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H24" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I24" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J24" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K24" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>146</v>
+        <v>26</v>
       </c>
       <c r="C25" t="s">
-        <v>147</v>
+        <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="E25">
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>149</v>
+        <v>28</v>
       </c>
       <c r="G25" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H25" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I25" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J25" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K25" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="G26" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H26" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I26" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J26" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K26" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
-        <v>153</v>
+        <v>104</v>
       </c>
       <c r="C27" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="D27" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="G27" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H27" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I27" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J27" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K27" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="B28" t="s">
-        <v>156</v>
+        <v>107</v>
       </c>
       <c r="C28" t="s">
-        <v>157</v>
+        <v>108</v>
       </c>
       <c r="D28" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="E28">
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="G28" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H28" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="I28" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="J28" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="K28" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2415,7 +3141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2424,23 +3150,23 @@
     <col min="4" max="4" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>161</v>
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="B2">
         <v>27</v>
@@ -2449,12 +3175,12 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="B3">
         <v>27</v>
@@ -2463,12 +3189,12 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>125</v>
       </c>
       <c r="B4">
         <v>32</v>
@@ -2477,12 +3203,12 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="B5">
         <v>52</v>
@@ -2491,12 +3217,12 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="B6">
         <v>27</v>
@@ -2505,12 +3231,12 @@
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>126</v>
       </c>
       <c r="B7">
         <v>8</v>
@@ -2519,12 +3245,12 @@
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="B8">
         <v>45</v>
@@ -2533,12 +3259,12 @@
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="B9">
         <v>31</v>
@@ -2547,12 +3273,12 @@
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="B10">
         <v>35</v>
@@ -2561,12 +3287,12 @@
         <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="B11">
         <v>12</v>
@@ -2575,12 +3301,12 @@
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B12">
         <v>53</v>
@@ -2589,12 +3315,12 @@
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B13">
         <v>18</v>
@@ -2603,12 +3329,12 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="B14">
         <v>9</v>
@@ -2617,7 +3343,7 @@
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2626,7 +3352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2635,196 +3361,196 @@
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>176</v>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="B2" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>135</v>
       </c>
       <c r="B3" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="B5" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B6" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="B7" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B8" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="B9" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>69</v>
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="B14" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>125</v>
       </c>
       <c r="B15" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="B20" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="B21" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="B22" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="B25" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>